<commit_message>
[update] stage4, stage5 구현
stage4, stage5 데이터 및 맵 구현
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Stage.xlsx
+++ b/JsonConverter/ExcelFiles/Stage.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OZ_Project\MinHyeong2DProject\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0106307-DC52-4310-9D17-981CD709642D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A92E8BCD-8405-42EB-9869-F78E81D3F5CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -97,11 +97,11 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>wave5_01, wave5_02, wave5_03</t>
+    <t>wave4_01, wave4_02, wave4_03, wave4_04, wave4_05</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>wave4_01, wave4_02, wave4_03</t>
+    <t>wave5_01, wave5_02, wave5_03, wave5_04, wave5_05, wave5_06, wave5_07, wave5_08</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -529,7 +529,8 @@
   <cols>
     <col min="1" max="1" width="19.42578125" style="2" customWidth="1"/>
     <col min="2" max="2" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="32.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="88.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="26.5703125" style="2" customWidth="1"/>
     <col min="7" max="8" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
@@ -687,7 +688,7 @@
         <v>200</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -712,7 +713,7 @@
         <v>200</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>

</xml_diff>